<commit_message>
Add email service tests and verify basic functionality
Co-authored-by: natalilerner-oss <244393048+natalilerner-oss@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test_portfolio_ישראלי_2024-01-15.xlsx
+++ b/test_portfolio_ישראלי_2024-01-15.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ביטוח" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="השוואת פוליסות" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="תחזיות פרמיה" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ביטוח" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="סיכום" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="השוואת פוליסות" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="תחזיות פרמיה" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -72,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -84,6 +84,10 @@
     </xf>
     <xf numFmtId="166" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -170,13 +174,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -200,7 +204,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -228,8 +232,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -255,8 +259,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -282,7 +286,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -297,9 +301,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -989,92 +993,140 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>כיסוי</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>12345678</t>
+          <t>12345678 (הראל)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>87654321</t>
+          <t>87654321 (פניקס)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>11223344</t>
+          <t>11223344 (מגדל)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>55667788</t>
+          <t>55667788 (כלל)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>99001122</t>
+          <t>99001122 (הראל)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>בריאות - ניתוחים שקל ראשון</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>101.04</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>89.5</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>156.75</v>
+          <t>אכ"ע</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="E2" s="3" t="n">
         <v>67.2</v>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>45.3</v>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>בריאות - תרופות מיוחדות</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>24.35</v>
+          <t>ביטוח חיים</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>156.75</v>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>בריאות - השתלות וטיפולים בחו"ל</t>
+          <t>השתלות וטיפולים בחו"ל</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
         <v>19.7</v>
       </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1082,26 +1134,145 @@
           <t>מחלות קשות</t>
         </is>
       </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ביטוח חיים</t>
+          <t>ניתוחים שקל ראשון</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>101.04</v>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>אכ"ע</t>
-        </is>
+          <t>תאונות אישיות</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>45.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>תאונות אישיות</t>
-        </is>
+          <t>תרופות מיוחדות</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>24.35</v>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>סה"כ</t>
+        </is>
+      </c>
+      <c r="B9" s="5">
+        <f>SUM(B2:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>SUM(C2:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="5">
+        <f>SUM(D2:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="5">
+        <f>SUM(E2:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>SUM(F2:F8)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>